<commit_message>
single stock analysis and autocallable notes
</commit_message>
<xml_diff>
--- a/epsilon-phi-core/src/Scripts/Case Studies/2. Optimizations/Simple Analysis.xlsx
+++ b/epsilon-phi-core/src/Scripts/Case Studies/2. Optimizations/Simple Analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/Repositories/Python/epsilon-phi/epsilon-phi-core/src/Scripts/Case Studies/2. Optimizations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{036B9071-05C5-8043-AE6A-14E0363FB6A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F38ABA85-6FEF-CE46-BCEB-528E5AA0F1B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="20320" windowHeight="19040" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1360" yWindow="500" windowWidth="20320" windowHeight="19040" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portfolios" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="146">
   <si>
     <t>Low Volatility</t>
   </si>
@@ -473,6 +473,12 @@
   </si>
   <si>
     <t>HFRIFFD</t>
+  </si>
+  <si>
+    <t>US Inflation Protected Bonds</t>
+  </si>
+  <si>
+    <t>MLG5QIL</t>
   </si>
 </sst>
 </file>
@@ -815,7 +821,7 @@
     </xf>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1102,6 +1108,9 @@
     </xf>
     <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5059,232 +5068,232 @@
   <sheetData>
     <row r="1" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="49"/>
-      <c r="B1" s="114" t="s">
+      <c r="B1" s="115" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114" t="s">
+      <c r="C1" s="115"/>
+      <c r="D1" s="115" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="114"/>
-      <c r="F1" s="114" t="s">
+      <c r="E1" s="115"/>
+      <c r="F1" s="115" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="114"/>
-      <c r="H1" s="114" t="s">
+      <c r="G1" s="115"/>
+      <c r="H1" s="115" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="115"/>
+      <c r="I1" s="116"/>
     </row>
     <row r="2" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="116">
+      <c r="B2" s="117">
         <v>0.745</v>
       </c>
-      <c r="C2" s="116"/>
-      <c r="D2" s="116" t="s">
+      <c r="C2" s="117"/>
+      <c r="D2" s="117" t="s">
         <v>38</v>
       </c>
-      <c r="E2" s="116"/>
-      <c r="F2" s="116">
+      <c r="E2" s="117"/>
+      <c r="F2" s="117">
         <v>0.36</v>
       </c>
-      <c r="G2" s="116"/>
-      <c r="H2" s="116">
+      <c r="G2" s="117"/>
+      <c r="H2" s="117">
         <v>0.15</v>
       </c>
-      <c r="I2" s="116"/>
+      <c r="I2" s="117"/>
     </row>
     <row r="3" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="109">
+      <c r="B3" s="110">
         <v>0.02</v>
       </c>
-      <c r="C3" s="109"/>
-      <c r="D3" s="109">
+      <c r="C3" s="110"/>
+      <c r="D3" s="110">
         <v>0.03</v>
       </c>
-      <c r="E3" s="109"/>
-      <c r="F3" s="109">
+      <c r="E3" s="110"/>
+      <c r="F3" s="110">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="G3" s="109"/>
-      <c r="H3" s="109">
+      <c r="G3" s="110"/>
+      <c r="H3" s="110">
         <v>5.5E-2</v>
       </c>
-      <c r="I3" s="109"/>
+      <c r="I3" s="110"/>
     </row>
     <row r="4" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="109">
+      <c r="B4" s="110">
         <v>0.14000000000000001</v>
       </c>
-      <c r="C4" s="109"/>
-      <c r="D4" s="109">
+      <c r="C4" s="110"/>
+      <c r="D4" s="110">
         <v>0.22500000000000001</v>
       </c>
-      <c r="E4" s="109"/>
-      <c r="F4" s="109">
+      <c r="E4" s="110"/>
+      <c r="F4" s="110">
         <v>0.35499999999999998</v>
       </c>
-      <c r="G4" s="109"/>
-      <c r="H4" s="109">
+      <c r="G4" s="110"/>
+      <c r="H4" s="110">
         <v>0.505</v>
       </c>
-      <c r="I4" s="109"/>
+      <c r="I4" s="110"/>
     </row>
     <row r="5" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="109">
+      <c r="B5" s="110">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="C5" s="109"/>
-      <c r="D5" s="109">
+      <c r="C5" s="110"/>
+      <c r="D5" s="110">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="E5" s="109"/>
-      <c r="F5" s="109">
+      <c r="E5" s="110"/>
+      <c r="F5" s="110">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="G5" s="109"/>
-      <c r="H5" s="109">
+      <c r="G5" s="110"/>
+      <c r="H5" s="110">
         <v>0.03</v>
       </c>
-      <c r="I5" s="109"/>
+      <c r="I5" s="110"/>
     </row>
     <row r="6" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="109">
+      <c r="B6" s="110">
         <v>0.04</v>
       </c>
-      <c r="C6" s="109"/>
-      <c r="D6" s="109">
+      <c r="C6" s="110"/>
+      <c r="D6" s="110">
         <v>5.5E-2</v>
       </c>
-      <c r="E6" s="109"/>
-      <c r="F6" s="109">
+      <c r="E6" s="110"/>
+      <c r="F6" s="110">
         <v>0.12</v>
       </c>
-      <c r="G6" s="109"/>
-      <c r="H6" s="109">
+      <c r="G6" s="110"/>
+      <c r="H6" s="110">
         <v>0.185</v>
       </c>
-      <c r="I6" s="109"/>
+      <c r="I6" s="110"/>
     </row>
     <row r="7" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="110">
+      <c r="B7" s="111">
         <v>0.04</v>
       </c>
-      <c r="C7" s="110"/>
-      <c r="D7" s="110">
+      <c r="C7" s="111"/>
+      <c r="D7" s="111">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="E7" s="110"/>
-      <c r="F7" s="110">
+      <c r="E7" s="111"/>
+      <c r="F7" s="111">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="G7" s="110"/>
-      <c r="H7" s="110">
+      <c r="G7" s="111"/>
+      <c r="H7" s="111">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="I7" s="110"/>
+      <c r="I7" s="111"/>
     </row>
     <row r="8" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="54" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="111">
+      <c r="B8" s="112">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="C8" s="111"/>
-      <c r="D8" s="111">
+      <c r="C8" s="112"/>
+      <c r="D8" s="112">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="E8" s="111"/>
-      <c r="F8" s="111">
+      <c r="E8" s="112"/>
+      <c r="F8" s="112">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G8" s="111"/>
-      <c r="H8" s="111">
+      <c r="G8" s="112"/>
+      <c r="H8" s="112">
         <v>7.5999999999999998E-2</v>
       </c>
-      <c r="I8" s="111"/>
+      <c r="I8" s="112"/>
     </row>
     <row r="9" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="54" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="112">
+      <c r="B9" s="113">
         <v>0.6</v>
       </c>
-      <c r="C9" s="112"/>
-      <c r="D9" s="112">
+      <c r="C9" s="113"/>
+      <c r="D9" s="113">
         <v>0.59</v>
       </c>
-      <c r="E9" s="112"/>
-      <c r="F9" s="112">
+      <c r="E9" s="113"/>
+      <c r="F9" s="113">
         <v>0.53</v>
       </c>
-      <c r="G9" s="112"/>
-      <c r="H9" s="112">
+      <c r="G9" s="113"/>
+      <c r="H9" s="113">
         <v>0.49</v>
       </c>
-      <c r="I9" s="112"/>
+      <c r="I9" s="113"/>
     </row>
     <row r="10" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="54" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="109">
+      <c r="B10" s="110">
         <v>3.1E-2</v>
       </c>
-      <c r="C10" s="109"/>
-      <c r="D10" s="109">
+      <c r="C10" s="110"/>
+      <c r="D10" s="110">
         <v>4.9000000000000002E-2</v>
       </c>
-      <c r="E10" s="109"/>
-      <c r="F10" s="109">
+      <c r="E10" s="110"/>
+      <c r="F10" s="110">
         <v>7.3999999999999996E-2</v>
       </c>
-      <c r="G10" s="109"/>
-      <c r="H10" s="109">
+      <c r="G10" s="110"/>
+      <c r="H10" s="110">
         <v>0.10299999999999999</v>
       </c>
-      <c r="I10" s="109"/>
+      <c r="I10" s="110"/>
     </row>
     <row r="11" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="B11" s="113" t="s">
+      <c r="B11" s="114" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="113"/>
-      <c r="D11" s="113" t="s">
+      <c r="C11" s="114"/>
+      <c r="D11" s="114" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="113"/>
-      <c r="F11" s="113" t="s">
+      <c r="E11" s="114"/>
+      <c r="F11" s="114" t="s">
         <v>34</v>
       </c>
-      <c r="G11" s="113"/>
-      <c r="H11" s="113" t="s">
+      <c r="G11" s="114"/>
+      <c r="H11" s="114" t="s">
         <v>35</v>
       </c>
-      <c r="I11" s="113"/>
+      <c r="I11" s="114"/>
     </row>
     <row r="12" spans="1:9" s="8" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="55" t="s">
@@ -5577,64 +5586,64 @@
       <c r="A23" s="58" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="107">
+      <c r="B23" s="108">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="C23" s="107"/>
-      <c r="D23" s="107">
+      <c r="C23" s="108"/>
+      <c r="D23" s="108">
         <v>3.7999999999999999E-2</v>
       </c>
-      <c r="E23" s="107"/>
-      <c r="F23" s="107">
+      <c r="E23" s="108"/>
+      <c r="F23" s="108">
         <v>6.3E-2</v>
       </c>
-      <c r="G23" s="107"/>
-      <c r="H23" s="107">
+      <c r="G23" s="108"/>
+      <c r="H23" s="108">
         <v>8.8999999999999996E-2</v>
       </c>
-      <c r="I23" s="107"/>
+      <c r="I23" s="108"/>
     </row>
     <row r="24" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="58" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="107">
+      <c r="B24" s="108">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="C24" s="107"/>
-      <c r="D24" s="107">
+      <c r="C24" s="108"/>
+      <c r="D24" s="108">
         <v>8.2000000000000003E-2</v>
       </c>
-      <c r="E24" s="107"/>
-      <c r="F24" s="107">
+      <c r="E24" s="108"/>
+      <c r="F24" s="108">
         <v>0.16200000000000001</v>
       </c>
-      <c r="G24" s="107"/>
-      <c r="H24" s="107">
+      <c r="G24" s="108"/>
+      <c r="H24" s="108">
         <v>0.24299999999999999</v>
       </c>
-      <c r="I24" s="107"/>
+      <c r="I24" s="108"/>
     </row>
     <row r="25" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="B25" s="108">
+      <c r="B25" s="109">
         <v>0</v>
       </c>
-      <c r="C25" s="108"/>
-      <c r="D25" s="108">
+      <c r="C25" s="109"/>
+      <c r="D25" s="109">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="E25" s="108"/>
-      <c r="F25" s="108">
+      <c r="E25" s="109"/>
+      <c r="F25" s="109">
         <v>0.14899999999999999</v>
       </c>
-      <c r="G25" s="108"/>
-      <c r="H25" s="108">
+      <c r="G25" s="109"/>
+      <c r="H25" s="109">
         <v>0.253</v>
       </c>
-      <c r="I25" s="108"/>
+      <c r="I25" s="109"/>
     </row>
     <row r="26" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="63" t="s">
@@ -5653,64 +5662,64 @@
       <c r="A27" s="58" t="s">
         <v>53</v>
       </c>
-      <c r="B27" s="107">
+      <c r="B27" s="108">
         <v>0.23799999999999999</v>
       </c>
-      <c r="C27" s="107"/>
-      <c r="D27" s="107">
+      <c r="C27" s="108"/>
+      <c r="D27" s="108">
         <v>0.27900000000000003</v>
       </c>
-      <c r="E27" s="107"/>
-      <c r="F27" s="107">
+      <c r="E27" s="108"/>
+      <c r="F27" s="108">
         <v>0.314</v>
       </c>
-      <c r="G27" s="107"/>
-      <c r="H27" s="107">
+      <c r="G27" s="108"/>
+      <c r="H27" s="108">
         <v>0.33700000000000002</v>
       </c>
-      <c r="I27" s="107"/>
+      <c r="I27" s="108"/>
     </row>
     <row r="28" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="58" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="107">
+      <c r="B28" s="108">
         <v>0.04</v>
       </c>
-      <c r="C28" s="107"/>
-      <c r="D28" s="107">
+      <c r="C28" s="108"/>
+      <c r="D28" s="108">
         <v>8.4000000000000005E-2</v>
       </c>
-      <c r="E28" s="107"/>
-      <c r="F28" s="107">
+      <c r="E28" s="108"/>
+      <c r="F28" s="108">
         <v>0.14299999999999999</v>
       </c>
-      <c r="G28" s="107"/>
-      <c r="H28" s="107">
+      <c r="G28" s="108"/>
+      <c r="H28" s="108">
         <v>0.187</v>
       </c>
-      <c r="I28" s="107"/>
+      <c r="I28" s="108"/>
     </row>
     <row r="29" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="107">
+      <c r="B29" s="108">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="C29" s="107"/>
-      <c r="D29" s="107">
+      <c r="C29" s="108"/>
+      <c r="D29" s="108">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="E29" s="107"/>
-      <c r="F29" s="107">
+      <c r="E29" s="108"/>
+      <c r="F29" s="108">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="G29" s="107"/>
-      <c r="H29" s="107">
+      <c r="G29" s="108"/>
+      <c r="H29" s="108">
         <v>0.108</v>
       </c>
-      <c r="I29" s="107"/>
+      <c r="I29" s="108"/>
     </row>
     <row r="30" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="55" t="s">
@@ -6767,16 +6776,16 @@
   <sheetData>
     <row r="1" spans="1:16" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="15"/>
-      <c r="B1" s="119" t="s">
+      <c r="B1" s="120" t="s">
         <v>96</v>
       </c>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
+      <c r="C1" s="120"/>
+      <c r="D1" s="120"/>
+      <c r="E1" s="120"/>
+      <c r="F1" s="120"/>
+      <c r="G1" s="120"/>
+      <c r="H1" s="120"/>
+      <c r="I1" s="120"/>
       <c r="J1" s="17"/>
       <c r="K1" s="3"/>
       <c r="L1" s="3"/>
@@ -6784,13 +6793,13 @@
     </row>
     <row r="2" spans="1:16" ht="41" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="18"/>
-      <c r="B2" s="117" t="s">
+      <c r="B2" s="118" t="s">
         <v>73</v>
       </c>
-      <c r="C2" s="117"/>
-      <c r="D2" s="118"/>
-      <c r="E2" s="118"/>
-      <c r="F2" s="118"/>
+      <c r="C2" s="118"/>
+      <c r="D2" s="119"/>
+      <c r="E2" s="119"/>
+      <c r="F2" s="119"/>
       <c r="G2" s="20" t="s">
         <v>31</v>
       </c>
@@ -7925,12 +7934,12 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D29E0093-E6C6-A248-AF2A-CA21312ABEE8}">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.6640625" style="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.5" style="1" bestFit="1" customWidth="1"/>
   </cols>
@@ -7939,7 +7948,7 @@
       <c r="A1" s="81" t="s">
         <v>115</v>
       </c>
-      <c r="B1" s="82" t="s">
+      <c r="B1" s="107" t="s">
         <v>123</v>
       </c>
       <c r="C1" s="82" t="s">
@@ -7988,10 +7997,10 @@
     </row>
     <row r="4" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
       <c r="B4" s="70" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="C4" s="70" t="s">
         <v>4</v>
@@ -8005,13 +8014,13 @@
     </row>
     <row r="5" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B5" s="70" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="C5" s="70" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D5" s="52">
         <v>0</v>
@@ -8022,10 +8031,10 @@
     </row>
     <row r="6" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B6" s="70" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="C6" s="70" t="s">
         <v>6</v>
@@ -8033,56 +8042,56 @@
       <c r="D6" s="52">
         <v>0</v>
       </c>
-      <c r="E6" s="52">
+      <c r="E6" s="31">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="B7" s="70" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="C7" s="70" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D7" s="52">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="E7" s="52">
-        <v>0.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
       <c r="B8" s="70" t="s">
-        <v>9</v>
+        <v>132</v>
       </c>
       <c r="C8" s="70" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="52">
-        <v>0.06</v>
-      </c>
-      <c r="E8" s="31">
-        <v>0</v>
+        <v>0.1</v>
+      </c>
+      <c r="E8" s="52">
+        <v>0.7</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B9" s="70" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C9" s="70" t="s">
         <v>8</v>
       </c>
       <c r="D9" s="52">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="E9" s="31">
         <v>0</v>
@@ -8090,16 +8099,16 @@
     </row>
     <row r="10" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B10" s="70" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C10" s="70" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="52">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="E10" s="31">
         <v>0</v>
@@ -8107,33 +8116,33 @@
     </row>
     <row r="11" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A11" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B11" s="70" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C11" s="70" t="s">
         <v>8</v>
       </c>
       <c r="D11" s="52">
-        <v>7.0000000000000007E-2</v>
+        <v>0</v>
       </c>
       <c r="E11" s="31">
-        <v>0.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B12" s="70" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C12" s="70" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="52">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E12" s="31">
         <v>0.7</v>
@@ -8141,16 +8150,16 @@
     </row>
     <row r="13" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B13" s="70" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C13" s="70" t="s">
         <v>8</v>
       </c>
       <c r="D13" s="52">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="E13" s="31">
         <v>0.7</v>
@@ -8158,61 +8167,61 @@
     </row>
     <row r="14" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B14" s="70" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C14" s="70" t="s">
         <v>8</v>
       </c>
       <c r="D14" s="52">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="E14" s="31">
         <v>0.7</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" s="12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B15" s="70" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C15" s="70" t="s">
         <v>8</v>
       </c>
       <c r="D15" s="52">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E15" s="31">
-        <v>0</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
-        <v>131</v>
+        <v>108</v>
       </c>
       <c r="B16" s="70" t="s">
-        <v>109</v>
+        <v>16</v>
       </c>
       <c r="C16" s="70" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="52">
+        <v>0.06</v>
+      </c>
+      <c r="E16" s="31">
         <v>0</v>
-      </c>
-      <c r="E16" s="85">
-        <v>0.7</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" s="12" t="s">
-        <v>111</v>
+        <v>131</v>
       </c>
       <c r="B17" s="70" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C17" s="70" t="s">
         <v>8</v>
@@ -8226,33 +8235,33 @@
     </row>
     <row r="18" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="12" t="s">
-        <v>143</v>
+        <v>111</v>
       </c>
       <c r="B18" s="70" t="s">
-        <v>142</v>
+        <v>110</v>
       </c>
       <c r="C18" s="70" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="D18" s="52">
-        <v>0.16</v>
-      </c>
-      <c r="E18" s="31">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="E18" s="85">
+        <v>0.7</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="12" t="s">
-        <v>112</v>
+        <v>143</v>
       </c>
       <c r="B19" s="70" t="s">
-        <v>18</v>
+        <v>142</v>
       </c>
       <c r="C19" s="70" t="s">
         <v>17</v>
       </c>
       <c r="D19" s="52">
-        <v>0</v>
+        <v>0.16</v>
       </c>
       <c r="E19" s="31">
         <v>1</v>
@@ -8260,10 +8269,10 @@
     </row>
     <row r="20" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B20" s="70" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C20" s="70" t="s">
         <v>17</v>
@@ -8277,10 +8286,10 @@
     </row>
     <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B21" s="70" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C21" s="70" t="s">
         <v>17</v>
@@ -8294,27 +8303,27 @@
     </row>
     <row r="22" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B22" s="70" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C22" s="70" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D22" s="52">
         <v>0</v>
       </c>
       <c r="E22" s="31">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" s="12" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="B23" s="70" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C23" s="70" t="s">
         <v>21</v>
@@ -8328,10 +8337,10 @@
     </row>
     <row r="24" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A24" s="12" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="B24" s="70" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C24" s="70" t="s">
         <v>21</v>
@@ -8345,13 +8354,13 @@
     </row>
     <row r="25" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A25" s="12" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B25" s="70" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C25" s="70" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D25" s="52">
         <v>0</v>
@@ -8362,10 +8371,10 @@
     </row>
     <row r="26" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A26" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B26" s="70" t="s">
-        <v>97</v>
+        <v>26</v>
       </c>
       <c r="C26" s="70" t="s">
         <v>25</v>
@@ -8379,10 +8388,10 @@
     </row>
     <row r="27" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A27" s="12" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B27" s="70" t="s">
-        <v>27</v>
+        <v>97</v>
       </c>
       <c r="C27" s="70" t="s">
         <v>25</v>
@@ -8395,16 +8404,33 @@
       </c>
     </row>
     <row r="28" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A28" s="80"/>
-      <c r="B28" s="78" t="s">
+      <c r="A28" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="B28" s="70" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" s="70" t="s">
+        <v>25</v>
+      </c>
+      <c r="D28" s="52">
+        <v>0</v>
+      </c>
+      <c r="E28" s="31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A29" s="80"/>
+      <c r="B29" s="78" t="s">
         <v>98</v>
       </c>
-      <c r="C28" s="78"/>
-      <c r="D28" s="86">
-        <f>SUM(D2:D27)</f>
+      <c r="C29" s="78"/>
+      <c r="D29" s="86">
+        <f>SUM(D2:D28)</f>
         <v>1</v>
       </c>
-      <c r="E28" s="79"/>
+      <c r="E29" s="79"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>